<commit_message>
data: 2026-07-14 일별 수집
</commit_message>
<xml_diff>
--- a/data/daily/2026-07/2026-07-14.xlsx
+++ b/data/daily/2026-07/2026-07-14.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="올리브영" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카테고리통계" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="카테고리통계" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,32 +439,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -770,7 +781,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>[그레인온] 골드 카무트 브랜드밀 효소 3개월(+선물포장)</t>
+          <t>[그레인온] 골드 카무트 브랜드밀 효소 3개월(+선물포장)+9포추가+파로저당견과류바+냉각선풍기 증정</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -860,22 +871,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>아메리카노 증정 에너지 활력선물 [김종국 추천세트]익스트림 아르기닌정 (2개월분) &amp; 밀크씨슬 플러스 (2개월분) + 쇼핑백 증정</t>
+          <t>[한끼통살] 단백질 든든형 닭가슴살 21일 식단관리+(증정)전자레인지 용기</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>익스트림</t>
+          <t>한끼통살</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>25,900원</t>
+          <t>33,000원</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/7556791</t>
+          <t>https://gift.kakao.com/product/12860133</t>
         </is>
       </c>
     </row>
@@ -890,22 +901,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>[한끼통살] 단백질 든든형 닭가슴살 21일 식단관리+(증정)전자레인지 용기</t>
+          <t>아르기닌 증정 남친 활력선물 대한민국 NO.1 김종국 트리플아르기닌 6200 (30포) + 아르기닌 추가 증정</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>한끼통살</t>
+          <t>익스트림</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>33,000원</t>
+          <t>45,000원</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/12860133</t>
+          <t>https://gift.kakao.com/product/7417420</t>
         </is>
       </c>
     </row>
@@ -920,7 +931,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>아르기닌 증정 남친 활력선물 대한민국 NO.1 김종국 트리플아르기닌 6200 (30포) + 아르기닌 추가 증정</t>
+          <t>아메리카노 증정 에너지 활력선물 [김종국 추천세트]익스트림 아르기닌정 (2개월분) &amp; 밀크씨슬 플러스 (2개월분) + 쇼핑백 증정</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -930,12 +941,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>45,000원</t>
+          <t>25,900원</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/7417420</t>
+          <t>https://gift.kakao.com/product/7556791</t>
         </is>
       </c>
     </row>
@@ -1073,41 +1084,41 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -1124,29 +1135,29 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[김우빈 PICK] 종근당건강 아임비타 비타민B 2000 30정 30일분</t>
+          <t>[의약외품][신혜선 PICK] 동국제약 멜라케어 더블 화이트 정 10정 10일분</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>종근당건강</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>3,000원</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=591581091&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610911058&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>루테인/눈건강</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1154,29 +1165,29 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>토비콤 루테인 지아잔틴 미니 30캡슐</t>
+          <t>[의약외품][신혜선 PICK] 동국 벤포 비타맥스정 10정 10일분</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>안국약품</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>2,000원</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=611982831&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610911056&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>혈행</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1184,29 +1195,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[다영 PICK] 셀트리온 다이어트 한 잔 슬림 S 프레소 10포 5일분</t>
+          <t>코엔자임 Q10 30캡슐 30일분</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2,000원</t>
+          <t>5,000원</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=944863413&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000144&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>루테인/눈건강</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1214,29 +1225,29 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>루테인 30정 30일분</t>
+          <t>[신혜선 PICK] 동국 마이팝 푸룬＆식이섬유</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>2,000원</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000126&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610911029&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>혈행</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1244,22 +1255,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>코엔자임 Q10 30캡슐 30일분</t>
+          <t>[다영 PICK] 셀트리온 다이어트 한 잔 슬림 S 프레소 10포 5일분</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>2,000원</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000144&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=944863413&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1274,12 +1285,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>비비랩 애사비 탱글 포켓 젤리 사과맛 5포 5일분</t>
+          <t>동국 맛있는 센시안 브이캔디 20정 20일분</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>비비랩 (BB LAB)</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1289,14 +1300,14 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=994852703&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910968&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>비타민D</t>
+          <t>루테인/눈건강</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1304,7 +1315,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>칼슘 마그네슘 비타민D 60정 30일분</t>
+          <t>루테인 30정 30일분</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1314,19 +1325,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>3,000원</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000148&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000126&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>마그네슘</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1334,7 +1345,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>철분 30정 30일분</t>
+          <t>마그네슘 30정 30일분</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1349,7 +1360,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000133&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000128&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1375,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>콜린 미오이노시톨 4000 10포</t>
+          <t>푸응 7days 팻버닝 21캡슐</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>안국약품</t>
+          <t>닥터블릿</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1379,14 +1390,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=985472642&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=613602085&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>멀티비타민/종합비타민</t>
+          <t>루테인/눈건강</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1394,12 +1405,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>[김우빈 PICK] 종근당건강 아임비타 멀티비타민 컴팩트 30정 30일분</t>
+          <t>rTG 오메가3 30캡슐 30일분</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>종근당건강</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1409,7 +1420,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=591581101&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000145&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1419,360 +1430,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>카테고리</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>순위</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>상품명</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>가격</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>상품URL</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>기타/특수목적</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>[올영단독/온열안대증정] 슬리플러스X카카오프렌즈 슬리핑보틀 100ml (1개입 /4개입 기획/6개입)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>슬리플러스</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>15,000원</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000259811&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>기타/특수목적</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>온리추얼 리셋 브이라인 7포 (+1포 증정) (8일분)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>온리추얼</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>17,900원</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000249190&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=2</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>다이어트/체중관리</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>[웰니스 루틴] 온리추얼 슬리밍컷 다이어트/리셋 브이라인/글로우업 콜라겐 7포(+1포)/14포 (8/14일분)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>온리추얼</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>16,900원</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000236701&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=3</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>피부/미용</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>[윤광UP]온리추얼 글로우업 글루타치온 콜라겐 7포 (+1포 증정)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>온리추얼</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>16,900원</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000247570&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=4</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>피부/미용</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>[리뷰이벤트/10일콜라겐/모공,목주름/PDRN] 라이필 더마콜라겐 시그니처RN (10일분)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>라이필</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>15,840원</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000259411&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>다이어트/체중관리</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>6</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>프로뉴트리션 듀얼플랜 다이어트 유산균 14포</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>프로뉴트리션</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>34,010원</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000205496&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=6</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>기타/특수목적</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>7</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>[7월 올영픽/파격특가] 멜라메이트 구미/로우슈가/버라이어티팩 구미 20/40/50구미</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>멜라메이트</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>12,900원</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000223554&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=7</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>기타/특수목적</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>8</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>[7월 올영픽/1일 1정] 바이탈뷰티 메타그린 슬림업 30일 (+15일)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>바이탈뷰티</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>26,900원</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000248462&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=8</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>기타/특수목적</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>9</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>[3+1] 내츄럴플러스 수용성 파워 커큐민 30정 1박스 (1개월분) / 3박스 구매 시 1박스 증정</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>내츄럴플러스</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>14,300원</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=B000000228959&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=9</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>프로바이오틱스/유산균</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>[덴프스] 덴마크 유산균이야기 우먼 2개월분(질유산균) + 철분 헤모케어 3포 증정</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>덴프스</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>37,050원</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000202658&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=10</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1790,32 +1447,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>비율(%)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>카카오선물하기</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>다이소몰</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>올리브영</t>
         </is>
@@ -1828,16 +1485,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>22.5</v>
+        <v>26.7</v>
       </c>
       <c r="D2" t="n">
         <v>8</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -1872,16 +1529,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -1894,16 +1551,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -1919,7 +1576,7 @@
         <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>6.7</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -1941,7 +1598,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>2.5</v>
+        <v>3.3</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -1963,7 +1620,7 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>2.5</v>
+        <v>3.3</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -1982,10 +1639,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>25</v>
+        <v>26.7</v>
       </c>
       <c r="D9" t="n">
         <v>7</v>
@@ -1994,7 +1651,7 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -2004,10 +1661,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -2016,7 +1673,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -2026,10 +1683,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>7.5</v>
+        <v>3.3</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -2038,7 +1695,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -2048,19 +1705,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
-        <v>30</v>
+        <v>26.7</v>
       </c>
       <c r="D12" t="n">
         <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -2070,7 +1727,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C13" t="n">
         <v>100</v>
@@ -2082,7 +1739,7 @@
         <v>10</v>
       </c>
       <c r="F13" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>